<commit_message>
Refactor code structure for improved readability and maintainability Added and adjusted sesonal prayers
</commit_message>
<xml_diff>
--- a/Tables.xlsx
+++ b/Tables.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="868" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="868" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المناسبات" sheetId="1" state="visible" r:id="rId1"/>
@@ -28,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -136,6 +136,14 @@
       <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="21">
@@ -529,7 +537,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -732,6 +740,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1368,7 +1382,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U29"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="17.85546875" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="17.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="4.42578125" bestFit="1" customWidth="1" style="70" min="1" max="1"/>
     <col width="12.28515625" bestFit="1" customWidth="1" style="70" min="2" max="2"/>
@@ -1383,8 +1397,8 @@
     <col width="11.140625" customWidth="1" style="70" min="11" max="11"/>
     <col width="17.85546875" customWidth="1" style="70" min="12" max="12"/>
     <col width="28" customWidth="1" style="70" min="13" max="13"/>
-    <col width="17.85546875" customWidth="1" style="70" min="14" max="97"/>
-    <col width="17.85546875" customWidth="1" style="70" min="98" max="16384"/>
+    <col width="17.85546875" customWidth="1" style="70" min="14" max="105"/>
+    <col width="17.85546875" customWidth="1" style="70" min="106" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="23.25" customHeight="1" s="55">
@@ -1418,23 +1432,23 @@
           <t>المناسبة</t>
         </is>
       </c>
-      <c r="I1" s="81" t="inlineStr">
+      <c r="I1" s="83" t="inlineStr">
         <is>
           <t>دور القمر</t>
         </is>
       </c>
-      <c r="J1" s="81" t="inlineStr">
+      <c r="J1" s="83" t="inlineStr">
         <is>
           <t>الفصح</t>
         </is>
       </c>
-      <c r="K1" s="80" t="n"/>
-      <c r="M1" s="91" t="inlineStr">
+      <c r="K1" s="82" t="n"/>
+      <c r="M1" s="93" t="inlineStr">
         <is>
           <t>السنة القبطية الحالية</t>
         </is>
       </c>
-      <c r="N1" s="80" t="n"/>
+      <c r="N1" s="82" t="n"/>
       <c r="R1" s="1" t="n"/>
     </row>
     <row r="2" ht="23.25" customHeight="1" s="55">
@@ -1461,21 +1475,21 @@
           <t>النيروز</t>
         </is>
       </c>
-      <c r="I2" s="82" t="n"/>
-      <c r="J2" s="81" t="inlineStr">
+      <c r="I2" s="84" t="n"/>
+      <c r="J2" s="83" t="inlineStr">
         <is>
           <t>اليوم</t>
         </is>
       </c>
-      <c r="K2" s="81" t="inlineStr">
+      <c r="K2" s="83" t="inlineStr">
         <is>
           <t>الشهر</t>
         </is>
       </c>
-      <c r="M2" s="79" t="n">
-        <v>1741</v>
-      </c>
-      <c r="N2" s="80" t="n"/>
+      <c r="M2" s="81" t="n">
+        <v>1742</v>
+      </c>
+      <c r="N2" s="82" t="n"/>
       <c r="R2" s="2" t="n"/>
     </row>
     <row r="3" ht="18.75" customHeight="1" s="55">
@@ -1587,12 +1601,12 @@
       <c r="K5" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="M5" s="85" t="inlineStr">
+      <c r="M5" s="87" t="inlineStr">
         <is>
           <t>لضمان عمل البرنامج بشكل صحيح لا تُغيّر أي شئ يدويًا في الملف</t>
         </is>
       </c>
-      <c r="N5" s="86" t="n"/>
+      <c r="N5" s="88" t="n"/>
       <c r="R5" s="5" t="n"/>
       <c r="T5" s="6" t="n"/>
     </row>
@@ -1629,8 +1643,8 @@
       <c r="K6" s="27" t="n">
         <v>7</v>
       </c>
-      <c r="M6" s="87" t="n"/>
-      <c r="N6" s="88" t="n"/>
+      <c r="M6" s="89" t="n"/>
+      <c r="N6" s="90" t="n"/>
       <c r="R6" s="5" t="n"/>
       <c r="T6" s="6" t="n"/>
     </row>
@@ -1651,7 +1665,7 @@
         <v/>
       </c>
       <c r="F7" s="37" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G7" s="38" t="inlineStr">
         <is>
@@ -1667,8 +1681,8 @@
       <c r="K7" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="M7" s="87" t="n"/>
-      <c r="N7" s="88" t="n"/>
+      <c r="M7" s="89" t="n"/>
+      <c r="N7" s="90" t="n"/>
       <c r="R7" s="5" t="n"/>
       <c r="T7" s="6" t="n"/>
     </row>
@@ -1705,8 +1719,8 @@
       <c r="K8" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="M8" s="87" t="n"/>
-      <c r="N8" s="88" t="n"/>
+      <c r="M8" s="89" t="n"/>
+      <c r="N8" s="90" t="n"/>
       <c r="R8" s="5" t="n"/>
       <c r="T8" s="6" t="n"/>
     </row>
@@ -1743,8 +1757,8 @@
       <c r="K9" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="M9" s="87" t="n"/>
-      <c r="N9" s="88" t="n"/>
+      <c r="M9" s="89" t="n"/>
+      <c r="N9" s="90" t="n"/>
       <c r="R9" s="5" t="n"/>
       <c r="T9" s="6" t="n"/>
     </row>
@@ -1781,8 +1795,8 @@
       <c r="K10" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="M10" s="87" t="n"/>
-      <c r="N10" s="88" t="n"/>
+      <c r="M10" s="89" t="n"/>
+      <c r="N10" s="90" t="n"/>
       <c r="R10" s="5" t="n"/>
       <c r="T10" s="6" t="n"/>
     </row>
@@ -1796,14 +1810,14 @@
         </is>
       </c>
       <c r="D11" s="35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E11" s="36">
         <f>VLOOKUP(D11, $A$2:$B$100, 2, FALSE)</f>
         <v/>
       </c>
       <c r="F11" s="37" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="G11" s="38" t="inlineStr">
         <is>
@@ -1819,8 +1833,8 @@
       <c r="K11" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="M11" s="87" t="n"/>
-      <c r="N11" s="88" t="n"/>
+      <c r="M11" s="89" t="n"/>
+      <c r="N11" s="90" t="n"/>
       <c r="R11" s="5" t="n"/>
       <c r="T11" s="6" t="n"/>
     </row>
@@ -1834,14 +1848,14 @@
         </is>
       </c>
       <c r="D12" s="35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E12" s="36">
         <f>VLOOKUP(D12, $A$2:$B$100, 2, FALSE)</f>
         <v/>
       </c>
       <c r="F12" s="37" t="n">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="G12" s="38" t="inlineStr">
         <is>
@@ -1857,8 +1871,8 @@
       <c r="K12" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="M12" s="87" t="n"/>
-      <c r="N12" s="88" t="n"/>
+      <c r="M12" s="89" t="n"/>
+      <c r="N12" s="90" t="n"/>
       <c r="R12" s="5" t="n"/>
       <c r="T12" s="6" t="n"/>
     </row>
@@ -1879,7 +1893,7 @@
         <v/>
       </c>
       <c r="F13" s="37" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="G13" s="38" t="inlineStr">
         <is>
@@ -1895,8 +1909,8 @@
       <c r="K13" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="M13" s="87" t="n"/>
-      <c r="N13" s="88" t="n"/>
+      <c r="M13" s="89" t="n"/>
+      <c r="N13" s="90" t="n"/>
       <c r="R13" s="5" t="n"/>
       <c r="T13" s="6" t="n"/>
     </row>
@@ -1933,8 +1947,8 @@
       <c r="K14" s="27" t="n">
         <v>7</v>
       </c>
-      <c r="M14" s="87" t="n"/>
-      <c r="N14" s="88" t="n"/>
+      <c r="M14" s="89" t="n"/>
+      <c r="N14" s="90" t="n"/>
       <c r="R14" s="5" t="n"/>
       <c r="T14" s="6" t="n"/>
     </row>
@@ -1963,21 +1977,21 @@
       <c r="K15" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="M15" s="87" t="n"/>
-      <c r="N15" s="88" t="n"/>
+      <c r="M15" s="89" t="n"/>
+      <c r="N15" s="90" t="n"/>
       <c r="R15" s="5" t="n"/>
       <c r="T15" s="6" t="n"/>
     </row>
     <row r="16" ht="18.75" customHeight="1" s="55">
       <c r="D16" s="35" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E16" s="36">
         <f>VLOOKUP(D16, $A$2:$B$100, 2, FALSE)</f>
         <v/>
       </c>
       <c r="F16" s="37" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="G16" s="38" t="inlineStr">
         <is>
@@ -1993,21 +2007,21 @@
       <c r="K16" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="M16" s="87" t="n"/>
-      <c r="N16" s="88" t="n"/>
+      <c r="M16" s="89" t="n"/>
+      <c r="N16" s="90" t="n"/>
       <c r="R16" s="5" t="n"/>
       <c r="T16" s="6" t="n"/>
     </row>
     <row r="17" ht="18.75" customHeight="1" s="55" thickBot="1">
       <c r="D17" s="35" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E17" s="36">
         <f>VLOOKUP(D17, $A$2:$B$100, 2, FALSE)</f>
         <v/>
       </c>
       <c r="F17" s="37" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="G17" s="38" t="inlineStr">
         <is>
@@ -2023,21 +2037,21 @@
       <c r="K17" s="27" t="n">
         <v>7</v>
       </c>
-      <c r="M17" s="89" t="n"/>
-      <c r="N17" s="90" t="n"/>
+      <c r="M17" s="91" t="n"/>
+      <c r="N17" s="92" t="n"/>
       <c r="R17" s="5" t="n"/>
       <c r="T17" s="6" t="n"/>
     </row>
     <row r="18" ht="18.75" customHeight="1" s="55" thickTop="1">
       <c r="D18" s="35" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E18" s="36">
         <f>VLOOKUP(D18, $A$2:$B$100, 2, FALSE)</f>
         <v/>
       </c>
       <c r="F18" s="37" t="n">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="G18" s="38" t="inlineStr">
         <is>
@@ -2066,7 +2080,7 @@
         <v/>
       </c>
       <c r="F19" s="37" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G19" s="38" t="inlineStr">
         <is>
@@ -2095,7 +2109,7 @@
         <v/>
       </c>
       <c r="F20" s="37" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G20" s="38" t="inlineStr">
         <is>
@@ -2124,7 +2138,7 @@
         <v/>
       </c>
       <c r="F21" s="37" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="G21" s="38" t="inlineStr">
         <is>
@@ -2153,7 +2167,7 @@
         <v/>
       </c>
       <c r="F22" s="37" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G22" s="38" t="inlineStr">
         <is>
@@ -2179,17 +2193,17 @@
           <t>دخول السيد المسيح إلى أرض مصر</t>
         </is>
       </c>
-      <c r="I23" s="83" t="inlineStr">
+      <c r="I23" s="85" t="inlineStr">
         <is>
           <t>دور القمر في السنة الحالية</t>
         </is>
       </c>
-      <c r="J23" s="84" t="inlineStr">
+      <c r="J23" s="86" t="inlineStr">
         <is>
           <t>الفصح في السنة الحالية</t>
         </is>
       </c>
-      <c r="K23" s="80" t="n"/>
+      <c r="K23" s="82" t="n"/>
     </row>
     <row r="24" ht="21" customHeight="1" s="55">
       <c r="D24" s="39" t="n">
@@ -2200,14 +2214,14 @@
         <v/>
       </c>
       <c r="F24" s="40" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="G24" s="41" t="inlineStr">
         <is>
           <t>عيد الصعود</t>
         </is>
       </c>
-      <c r="I24" s="82" t="n"/>
+      <c r="I24" s="84" t="n"/>
       <c r="J24" s="11" t="inlineStr">
         <is>
           <t>اليوم</t>
@@ -2221,14 +2235,14 @@
     </row>
     <row r="25" ht="21" customHeight="1" s="55">
       <c r="D25" s="39" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E25" s="36">
         <f>VLOOKUP(D25, $A$2:$B$100, 2, FALSE)</f>
         <v/>
       </c>
       <c r="F25" s="40" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="G25" s="41" t="inlineStr">
         <is>
@@ -2236,7 +2250,7 @@
         </is>
       </c>
       <c r="I25" s="12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J25" s="15">
         <f>VLOOKUP(I25,I3:J21, 2, FALSE)</f>
@@ -2351,7 +2365,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S51"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="70" min="1" max="1"/>
     <col width="15" customWidth="1" style="70" min="2" max="2"/>
@@ -2371,8 +2385,8 @@
     <col width="12.7109375" customWidth="1" style="70" min="17" max="17"/>
     <col width="13.85546875" customWidth="1" style="70" min="18" max="18"/>
     <col width="14.140625" customWidth="1" style="70" min="19" max="19"/>
-    <col width="9.140625" customWidth="1" style="70" min="20" max="51"/>
-    <col width="9.140625" customWidth="1" style="70" min="52" max="16384"/>
+    <col width="9.140625" customWidth="1" style="70" min="20" max="59"/>
+    <col width="9.140625" customWidth="1" style="70" min="60" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="54" customFormat="1" customHeight="1" s="44">
@@ -2474,7 +2488,7 @@
     </row>
     <row r="2">
       <c r="A2" s="45" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B2" s="45" t="n">
         <v>6</v>
@@ -2527,7 +2541,7 @@
     </row>
     <row r="3">
       <c r="A3" s="45" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B3" s="45" t="n">
         <v>6</v>
@@ -2586,7 +2600,7 @@
     </row>
     <row r="4">
       <c r="A4" s="45" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B4" s="45" t="n">
         <v>6</v>
@@ -2635,7 +2649,7 @@
     </row>
     <row r="5">
       <c r="A5" s="45" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B5" s="45" t="n">
         <v>6</v>
@@ -2680,7 +2694,7 @@
     </row>
     <row r="6">
       <c r="A6" s="45" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B6" s="45" t="n">
         <v>6</v>
@@ -2725,7 +2739,7 @@
     </row>
     <row r="7">
       <c r="A7" s="45" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B7" s="45" t="n">
         <v>6</v>
@@ -2770,7 +2784,7 @@
     </row>
     <row r="8">
       <c r="A8" s="45" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="B8" s="45" t="n">
         <v>6</v>
@@ -2815,7 +2829,7 @@
     </row>
     <row r="9">
       <c r="A9" s="45" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B9" s="45" t="n">
         <v>6</v>
@@ -2858,7 +2872,7 @@
     </row>
     <row r="10">
       <c r="A10" s="45" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B10" s="45" t="n">
         <v>6</v>
@@ -2917,7 +2931,7 @@
     </row>
     <row r="11">
       <c r="A11" s="45" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="B11" s="45" t="n">
         <v>6</v>
@@ -2962,7 +2976,7 @@
     </row>
     <row r="12">
       <c r="A12" s="45" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B12" s="45" t="n">
         <v>6</v>
@@ -3007,7 +3021,7 @@
     </row>
     <row r="13">
       <c r="A13" s="45" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="B13" s="45" t="n">
         <v>6</v>
@@ -3052,7 +3066,7 @@
     </row>
     <row r="14">
       <c r="A14" s="45" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B14" s="45" t="n">
         <v>6</v>
@@ -3097,7 +3111,7 @@
     </row>
     <row r="15">
       <c r="A15" s="45" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B15" s="45" t="n">
         <v>6</v>
@@ -3142,7 +3156,7 @@
     </row>
     <row r="16">
       <c r="A16" s="45" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B16" s="45" t="n">
         <v>6</v>
@@ -3185,7 +3199,7 @@
     </row>
     <row r="17">
       <c r="A17" s="45" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B17" s="45" t="n">
         <v>6</v>
@@ -3244,10 +3258,10 @@
     </row>
     <row r="18">
       <c r="A18" s="45" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="B18" s="45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C18" s="45" t="n"/>
       <c r="D18" s="45" t="n"/>
@@ -3289,10 +3303,10 @@
     </row>
     <row r="19">
       <c r="A19" s="45" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="B19" s="45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C19" s="45" t="n"/>
       <c r="D19" s="45" t="n"/>
@@ -3334,10 +3348,10 @@
     </row>
     <row r="20">
       <c r="A20" s="45" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B20" s="45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C20" s="45" t="n"/>
       <c r="D20" s="45" t="n"/>
@@ -3379,10 +3393,10 @@
     </row>
     <row r="21">
       <c r="A21" s="45" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="B21" s="45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C21" s="45" t="n"/>
       <c r="D21" s="45" t="n"/>
@@ -3424,10 +3438,10 @@
     </row>
     <row r="22">
       <c r="A22" s="45" t="n">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="B22" s="45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C22" s="45" t="n"/>
       <c r="D22" s="45" t="n"/>
@@ -3469,10 +3483,10 @@
     </row>
     <row r="23">
       <c r="A23" s="45" t="n">
+        <v>28</v>
+      </c>
+      <c r="B23" s="45" t="n">
         <v>6</v>
-      </c>
-      <c r="B23" s="45" t="n">
-        <v>7</v>
       </c>
       <c r="C23" s="45" t="n"/>
       <c r="D23" s="45" t="n"/>
@@ -3512,10 +3526,10 @@
     </row>
     <row r="24">
       <c r="A24" s="45" t="n">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="B24" s="45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C24" s="45" t="n">
         <v>1059</v>
@@ -3571,10 +3585,10 @@
     </row>
     <row r="25">
       <c r="A25" s="45" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="B25" s="45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C25" s="45" t="n"/>
       <c r="D25" s="45" t="n"/>
@@ -3616,7 +3630,7 @@
     </row>
     <row r="26">
       <c r="A26" s="45" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="B26" s="45" t="n">
         <v>7</v>
@@ -3661,7 +3675,7 @@
     </row>
     <row r="27">
       <c r="A27" s="45" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B27" s="45" t="n">
         <v>7</v>
@@ -3706,7 +3720,7 @@
     </row>
     <row r="28">
       <c r="A28" s="45" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B28" s="45" t="n">
         <v>7</v>
@@ -3751,7 +3765,7 @@
     </row>
     <row r="29">
       <c r="A29" s="45" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B29" s="45" t="n">
         <v>7</v>
@@ -3796,7 +3810,7 @@
     </row>
     <row r="30">
       <c r="A30" s="45" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="B30" s="45" t="n">
         <v>7</v>
@@ -3839,7 +3853,7 @@
     </row>
     <row r="31">
       <c r="A31" s="45" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B31" s="45" t="n">
         <v>7</v>
@@ -3898,7 +3912,7 @@
     </row>
     <row r="32">
       <c r="A32" s="45" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B32" s="45" t="n">
         <v>7</v>
@@ -3943,7 +3957,7 @@
     </row>
     <row r="33">
       <c r="A33" s="45" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B33" s="45" t="n">
         <v>7</v>
@@ -3988,7 +4002,7 @@
     </row>
     <row r="34">
       <c r="A34" s="45" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B34" s="45" t="n">
         <v>7</v>
@@ -4033,7 +4047,7 @@
     </row>
     <row r="35">
       <c r="A35" s="45" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B35" s="45" t="n">
         <v>7</v>
@@ -4078,7 +4092,7 @@
     </row>
     <row r="36">
       <c r="A36" s="45" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B36" s="45" t="n">
         <v>7</v>
@@ -4123,7 +4137,7 @@
     </row>
     <row r="37">
       <c r="A37" s="45" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B37" s="45" t="n">
         <v>7</v>
@@ -4166,7 +4180,7 @@
     </row>
     <row r="38">
       <c r="A38" s="45" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="B38" s="45" t="n">
         <v>7</v>
@@ -4225,7 +4239,7 @@
     </row>
     <row r="39">
       <c r="A39" s="45" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B39" s="45" t="n">
         <v>7</v>
@@ -4270,7 +4284,7 @@
     </row>
     <row r="40">
       <c r="A40" s="45" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B40" s="45" t="n">
         <v>7</v>
@@ -4315,7 +4329,7 @@
     </row>
     <row r="41">
       <c r="A41" s="45" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="B41" s="45" t="n">
         <v>7</v>
@@ -4360,7 +4374,7 @@
     </row>
     <row r="42">
       <c r="A42" s="45" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B42" s="45" t="n">
         <v>7</v>
@@ -4405,7 +4419,7 @@
     </row>
     <row r="43">
       <c r="A43" s="45" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="B43" s="45" t="n">
         <v>7</v>
@@ -4450,7 +4464,7 @@
     </row>
     <row r="44">
       <c r="A44" s="45" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B44" s="45" t="n">
         <v>7</v>
@@ -4493,7 +4507,7 @@
     </row>
     <row r="45">
       <c r="A45" s="45" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B45" s="45" t="n">
         <v>7</v>
@@ -4552,7 +4566,7 @@
     </row>
     <row r="46">
       <c r="A46" s="45" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B46" s="45" t="n">
         <v>7</v>
@@ -4597,7 +4611,7 @@
     </row>
     <row r="47">
       <c r="A47" s="45" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B47" s="45" t="n">
         <v>7</v>
@@ -4642,10 +4656,10 @@
     </row>
     <row r="48">
       <c r="A48" s="45" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="B48" s="45" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C48" s="45" t="n"/>
       <c r="D48" s="45" t="n"/>
@@ -4687,10 +4701,10 @@
     </row>
     <row r="49">
       <c r="A49" s="45" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="B49" s="45" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C49" s="45" t="n"/>
       <c r="D49" s="45" t="n"/>
@@ -4732,10 +4746,10 @@
     </row>
     <row r="50">
       <c r="A50" s="45" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B50" s="45" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C50" s="45" t="n"/>
       <c r="D50" s="45" t="n"/>
@@ -4777,10 +4791,10 @@
     </row>
     <row r="51">
       <c r="A51" s="45" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="B51" s="45" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C51" s="45" t="n"/>
       <c r="D51" s="45" t="n"/>
@@ -4837,7 +4851,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.42578125" bestFit="1" customWidth="1" style="55" min="1" max="1"/>
     <col width="7.7109375" bestFit="1" customWidth="1" style="55" min="2" max="2"/>
@@ -4971,10 +4985,10 @@
     </row>
     <row r="2" ht="23.25" customHeight="1" s="55">
       <c r="A2" s="48" t="n">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="B2" s="48" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C2" s="48" t="n">
         <v>1</v>
@@ -5046,8 +5060,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:I51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" bestFit="1" customWidth="1" style="55" min="1" max="1"/>
     <col width="15" bestFit="1" customWidth="1" style="55" min="2" max="2"/>
@@ -5056,53 +5070,59 @@
     <col width="12.7109375" bestFit="1" customWidth="1" style="55" min="5" max="5"/>
     <col width="9.28515625" bestFit="1" customWidth="1" style="55" min="7" max="7"/>
     <col width="15.140625" bestFit="1" customWidth="1" style="55" min="8" max="8"/>
+    <col width="11.28515625" bestFit="1" customWidth="1" style="70" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" customHeight="1" s="55">
-      <c r="A1" s="81" t="inlineStr">
+      <c r="A1" s="83" t="inlineStr">
         <is>
           <t>اليوم</t>
         </is>
       </c>
-      <c r="B1" s="81" t="inlineStr">
+      <c r="B1" s="83" t="inlineStr">
         <is>
           <t>الشهر</t>
         </is>
       </c>
-      <c r="C1" s="81" t="inlineStr">
+      <c r="C1" s="83" t="inlineStr">
         <is>
           <t xml:space="preserve">البولس </t>
         </is>
       </c>
-      <c r="D1" s="81" t="inlineStr">
+      <c r="D1" s="83" t="inlineStr">
         <is>
           <t>الكاثوليكون</t>
         </is>
       </c>
-      <c r="E1" s="81" t="inlineStr">
+      <c r="E1" s="83" t="inlineStr">
         <is>
           <t>الابركسيس</t>
         </is>
       </c>
-      <c r="F1" s="81" t="inlineStr">
+      <c r="F1" s="83" t="inlineStr">
         <is>
           <t>المزمور</t>
         </is>
       </c>
-      <c r="G1" s="81" t="inlineStr">
+      <c r="G1" s="83" t="inlineStr">
         <is>
           <t>الإنجيل</t>
         </is>
       </c>
-      <c r="H1" s="81" t="inlineStr">
+      <c r="H1" s="83" t="inlineStr">
         <is>
           <t>نهاية الانجيل</t>
         </is>
       </c>
-    </row>
-    <row r="2">
+      <c r="I1" s="79" t="inlineStr">
+        <is>
+          <t>ملاحظات</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" s="55">
       <c r="A2" s="8" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>8</v>
@@ -5125,10 +5145,15 @@
       <c r="H2" s="8" t="n">
         <v>35</v>
       </c>
+      <c r="I2" s="80" t="inlineStr">
+        <is>
+          <t>عيد القيامة</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="49" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="B3" s="49" t="n">
         <v>8</v>
@@ -5151,10 +5176,11 @@
       <c r="H3" s="49" t="n">
         <v>64</v>
       </c>
+      <c r="I3" s="45" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="49" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B4" s="49" t="n">
         <v>8</v>
@@ -5177,10 +5203,11 @@
       <c r="H4" s="49" t="n">
         <v>87</v>
       </c>
+      <c r="I4" s="45" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="49" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B5" s="49" t="n">
         <v>8</v>
@@ -5203,10 +5230,11 @@
       <c r="H5" s="49" t="n">
         <v>108</v>
       </c>
+      <c r="I5" s="45" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="49" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B6" s="49" t="n">
         <v>8</v>
@@ -5229,10 +5257,11 @@
       <c r="H6" s="49" t="n">
         <v>126</v>
       </c>
+      <c r="I6" s="45" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="49" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B7" s="49" t="n">
         <v>8</v>
@@ -5255,10 +5284,11 @@
       <c r="H7" s="49" t="n">
         <v>140</v>
       </c>
+      <c r="I7" s="45" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="49" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B8" s="49" t="n">
         <v>8</v>
@@ -5281,10 +5311,11 @@
       <c r="H8" s="49" t="n">
         <v>159</v>
       </c>
+      <c r="I8" s="45" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="49" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B9" s="49" t="n">
         <v>8</v>
@@ -5307,10 +5338,11 @@
       <c r="H9" s="49" t="n">
         <v>180</v>
       </c>
+      <c r="I9" s="45" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="49" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B10" s="49" t="n">
         <v>8</v>
@@ -5333,10 +5365,11 @@
       <c r="H10" s="49" t="n">
         <v>189</v>
       </c>
+      <c r="I10" s="45" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="49" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="B11" s="49" t="n">
         <v>8</v>
@@ -5359,10 +5392,11 @@
       <c r="H11" s="49" t="n">
         <v>198</v>
       </c>
+      <c r="I11" s="45" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="49" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B12" s="49" t="n">
         <v>8</v>
@@ -5385,10 +5419,11 @@
       <c r="H12" s="49" t="n">
         <v>209</v>
       </c>
+      <c r="I12" s="45" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="49" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B13" s="49" t="n">
         <v>8</v>
@@ -5411,10 +5446,11 @@
       <c r="H13" s="49" t="n">
         <v>220</v>
       </c>
+      <c r="I13" s="45" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="49" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="B14" s="49" t="n">
         <v>8</v>
@@ -5437,10 +5473,11 @@
       <c r="H14" s="49" t="n">
         <v>228</v>
       </c>
+      <c r="I14" s="45" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="49" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B15" s="49" t="n">
         <v>8</v>
@@ -5463,10 +5500,11 @@
       <c r="H15" s="49" t="n">
         <v>242</v>
       </c>
+      <c r="I15" s="45" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="49" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="B16" s="49" t="n">
         <v>8</v>
@@ -5489,10 +5527,11 @@
       <c r="H16" s="49" t="n">
         <v>260</v>
       </c>
+      <c r="I16" s="45" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="49" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B17" s="49" t="n">
         <v>8</v>
@@ -5515,10 +5554,11 @@
       <c r="H17" s="49" t="n">
         <v>268</v>
       </c>
+      <c r="I17" s="45" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="49" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B18" s="49" t="n">
         <v>8</v>
@@ -5541,10 +5581,11 @@
       <c r="H18" s="49" t="n">
         <v>281</v>
       </c>
+      <c r="I18" s="45" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="49" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B19" s="49" t="n">
         <v>8</v>
@@ -5567,10 +5608,11 @@
       <c r="H19" s="49" t="n">
         <v>290</v>
       </c>
+      <c r="I19" s="45" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="49" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B20" s="49" t="n">
         <v>8</v>
@@ -5593,13 +5635,14 @@
       <c r="H20" s="49" t="n">
         <v>300</v>
       </c>
+      <c r="I20" s="45" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="49" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="B21" s="49" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C21" s="49" t="n">
         <v>302</v>
@@ -5619,13 +5662,14 @@
       <c r="H21" s="49" t="n">
         <v>312</v>
       </c>
+      <c r="I21" s="45" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="49" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="B22" s="49" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C22" s="49" t="n">
         <v>314</v>
@@ -5645,13 +5689,14 @@
       <c r="H22" s="49" t="n">
         <v>328</v>
       </c>
+      <c r="I22" s="45" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="49" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B23" s="49" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C23" s="49" t="n">
         <v>330</v>
@@ -5671,13 +5716,14 @@
       <c r="H23" s="49" t="n">
         <v>358</v>
       </c>
+      <c r="I23" s="45" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="49" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="B24" s="49" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C24" s="49" t="n">
         <v>360</v>
@@ -5697,13 +5743,14 @@
       <c r="H24" s="49" t="n">
         <v>370</v>
       </c>
+      <c r="I24" s="45" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="49" t="n">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="B25" s="49" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C25" s="49" t="n">
         <v>372</v>
@@ -5723,13 +5770,14 @@
       <c r="H25" s="49" t="n">
         <v>378</v>
       </c>
+      <c r="I25" s="45" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="49" t="n">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="B26" s="49" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C26" s="49" t="n">
         <v>380</v>
@@ -5749,13 +5797,14 @@
       <c r="H26" s="49" t="n">
         <v>395</v>
       </c>
+      <c r="I26" s="45" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="49" t="n">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="B27" s="49" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C27" s="49" t="n">
         <v>397</v>
@@ -5775,13 +5824,14 @@
       <c r="H27" s="49" t="n">
         <v>407</v>
       </c>
+      <c r="I27" s="45" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="49" t="n">
+        <v>30</v>
+      </c>
+      <c r="B28" s="49" t="n">
         <v>8</v>
-      </c>
-      <c r="B28" s="49" t="n">
-        <v>9</v>
       </c>
       <c r="C28" s="49" t="n">
         <v>409</v>
@@ -5801,10 +5851,11 @@
       <c r="H28" s="49" t="n">
         <v>418</v>
       </c>
+      <c r="I28" s="45" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="49" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="B29" s="49" t="n">
         <v>9</v>
@@ -5827,10 +5878,11 @@
       <c r="H29" s="49" t="n">
         <v>437</v>
       </c>
+      <c r="I29" s="45" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="49" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B30" s="49" t="n">
         <v>9</v>
@@ -5853,10 +5905,11 @@
       <c r="H30" s="49" t="n">
         <v>458</v>
       </c>
+      <c r="I30" s="45" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="49" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B31" s="49" t="n">
         <v>9</v>
@@ -5879,10 +5932,11 @@
       <c r="H31" s="49" t="n">
         <v>470</v>
       </c>
+      <c r="I31" s="45" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="49" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B32" s="49" t="n">
         <v>9</v>
@@ -5905,10 +5959,11 @@
       <c r="H32" s="49" t="n">
         <v>481</v>
       </c>
+      <c r="I32" s="45" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="49" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="B33" s="49" t="n">
         <v>9</v>
@@ -5931,10 +5986,11 @@
       <c r="H33" s="49" t="n">
         <v>494</v>
       </c>
+      <c r="I33" s="45" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="49" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B34" s="49" t="n">
         <v>9</v>
@@ -5957,10 +6013,11 @@
       <c r="H34" s="49" t="n">
         <v>506</v>
       </c>
+      <c r="I34" s="45" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="49" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B35" s="49" t="n">
         <v>9</v>
@@ -5983,10 +6040,11 @@
       <c r="H35" s="49" t="n">
         <v>515</v>
       </c>
+      <c r="I35" s="45" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="49" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B36" s="49" t="n">
         <v>9</v>
@@ -6009,10 +6067,11 @@
       <c r="H36" s="49" t="n">
         <v>534</v>
       </c>
+      <c r="I36" s="45" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="49" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B37" s="49" t="n">
         <v>9</v>
@@ -6035,10 +6094,11 @@
       <c r="H37" s="49" t="n">
         <v>559</v>
       </c>
+      <c r="I37" s="45" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="49" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B38" s="49" t="n">
         <v>9</v>
@@ -6061,10 +6121,11 @@
       <c r="H38" s="49" t="n">
         <v>574</v>
       </c>
+      <c r="I38" s="45" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="49" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B39" s="49" t="n">
         <v>9</v>
@@ -6087,10 +6148,11 @@
       <c r="H39" s="49" t="n">
         <v>587</v>
       </c>
+      <c r="I39" s="45" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="49" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B40" s="49" t="n">
         <v>9</v>
@@ -6113,10 +6175,11 @@
       <c r="H40" s="49" t="n">
         <v>602</v>
       </c>
-    </row>
-    <row r="41">
+      <c r="I40" s="45" t="n"/>
+    </row>
+    <row r="41" ht="15.75" customHeight="1" s="55">
       <c r="A41" s="8" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="B41" s="8" t="n">
         <v>9</v>
@@ -6139,10 +6202,15 @@
       <c r="H41" s="8" t="n">
         <v>625</v>
       </c>
-    </row>
-    <row r="42">
+      <c r="I41" s="80" t="inlineStr">
+        <is>
+          <t>عيد الصعود</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="15.75" customHeight="1" s="55">
       <c r="A42" s="49" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B42" s="49" t="n">
         <v>9</v>
@@ -6165,10 +6233,11 @@
       <c r="H42" s="49" t="n">
         <v>643</v>
       </c>
-    </row>
-    <row r="43">
+      <c r="I42" s="80" t="n"/>
+    </row>
+    <row r="43" ht="15.75" customHeight="1" s="55">
       <c r="A43" s="49" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B43" s="49" t="n">
         <v>9</v>
@@ -6191,10 +6260,11 @@
       <c r="H43" s="49" t="n">
         <v>658</v>
       </c>
-    </row>
-    <row r="44">
+      <c r="I43" s="80" t="n"/>
+    </row>
+    <row r="44" ht="15.75" customHeight="1" s="55">
       <c r="A44" s="49" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="B44" s="49" t="n">
         <v>9</v>
@@ -6217,10 +6287,11 @@
       <c r="H44" s="49" t="n">
         <v>678</v>
       </c>
-    </row>
-    <row r="45">
+      <c r="I44" s="80" t="n"/>
+    </row>
+    <row r="45" ht="15.75" customHeight="1" s="55">
       <c r="A45" s="49" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B45" s="49" t="n">
         <v>9</v>
@@ -6243,10 +6314,11 @@
       <c r="H45" s="49" t="n">
         <v>694</v>
       </c>
-    </row>
-    <row r="46">
+      <c r="I45" s="80" t="n"/>
+    </row>
+    <row r="46" ht="15.75" customHeight="1" s="55">
       <c r="A46" s="49" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="B46" s="49" t="n">
         <v>9</v>
@@ -6269,10 +6341,11 @@
       <c r="H46" s="49" t="n">
         <v>707</v>
       </c>
-    </row>
-    <row r="47">
+      <c r="I46" s="80" t="n"/>
+    </row>
+    <row r="47" ht="15.75" customHeight="1" s="55">
       <c r="A47" s="49" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B47" s="49" t="n">
         <v>9</v>
@@ -6295,10 +6368,11 @@
       <c r="H47" s="49" t="n">
         <v>724</v>
       </c>
-    </row>
-    <row r="48">
+      <c r="I47" s="80" t="n"/>
+    </row>
+    <row r="48" ht="15.75" customHeight="1" s="55">
       <c r="A48" s="49" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B48" s="49" t="n">
         <v>9</v>
@@ -6321,10 +6395,11 @@
       <c r="H48" s="49" t="n">
         <v>740</v>
       </c>
-    </row>
-    <row r="49">
+      <c r="I48" s="80" t="n"/>
+    </row>
+    <row r="49" ht="15.75" customHeight="1" s="55">
       <c r="A49" s="49" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B49" s="49" t="n">
         <v>9</v>
@@ -6347,10 +6422,11 @@
       <c r="H49" s="49" t="n">
         <v>751</v>
       </c>
-    </row>
-    <row r="50">
+      <c r="I49" s="80" t="n"/>
+    </row>
+    <row r="50" ht="15.75" customHeight="1" s="55">
       <c r="A50" s="49" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B50" s="49" t="n">
         <v>9</v>
@@ -6373,13 +6449,14 @@
       <c r="H50" s="49" t="n">
         <v>777</v>
       </c>
-    </row>
-    <row r="51">
+      <c r="I50" s="80" t="n"/>
+    </row>
+    <row r="51" ht="15.75" customHeight="1" s="55">
       <c r="A51" s="8" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="B51" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C51" s="8" t="n">
         <v>779</v>
@@ -6398,6 +6475,11 @@
       </c>
       <c r="H51" s="8" t="n">
         <v>813</v>
+      </c>
+      <c r="I51" s="80" t="inlineStr">
+        <is>
+          <t>عيد العنصرة</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -9354,7 +9436,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P71"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" bestFit="1" customWidth="1" style="55" min="1" max="1"/>
     <col width="15" bestFit="1" customWidth="1" style="55" min="2" max="2"/>
@@ -12682,7 +12764,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E71"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.140625" customWidth="1" style="55" min="5" max="5"/>
   </cols>
@@ -15139,7 +15221,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H71"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.28515625" bestFit="1" customWidth="1" style="55" min="1" max="1"/>
     <col width="7.42578125" bestFit="1" customWidth="1" style="55" min="2" max="2"/>
@@ -17019,8 +17101,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:E50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.85546875" bestFit="1" customWidth="1" style="55" min="1" max="1"/>
     <col width="7.42578125" bestFit="1" customWidth="1" style="55" min="2" max="2"/>
@@ -17895,7 +17977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="21" customHeight="1" s="55">
@@ -18766,7 +18848,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H50"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.28515625" bestFit="1" customWidth="1" style="55" min="1" max="1"/>
     <col width="7.42578125" bestFit="1" customWidth="1" style="55" min="2" max="2"/>
@@ -20100,7 +20182,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.28515625" bestFit="1" customWidth="1" style="55" min="1" max="1"/>
     <col width="7.42578125" bestFit="1" customWidth="1" style="55" min="2" max="2"/>
@@ -20197,10 +20279,10 @@
     </row>
     <row r="2">
       <c r="A2" s="49" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B2" s="49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C2" s="49" t="n">
         <v>2</v>
@@ -20244,10 +20326,10 @@
     </row>
     <row r="3">
       <c r="A3" s="49" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="B3" s="49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3" s="49" t="inlineStr"/>
       <c r="D3" s="49" t="inlineStr"/>
@@ -20285,10 +20367,10 @@
     </row>
     <row r="4">
       <c r="A4" s="49" t="n">
+        <v>27</v>
+      </c>
+      <c r="B4" s="49" t="n">
         <v>5</v>
-      </c>
-      <c r="B4" s="49" t="n">
-        <v>6</v>
       </c>
       <c r="C4" s="49" t="inlineStr"/>
       <c r="D4" s="49" t="inlineStr"/>
@@ -20326,10 +20408,10 @@
     </row>
     <row r="5">
       <c r="A5" s="49" t="n">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="B5" s="49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C5" s="49" t="inlineStr"/>
       <c r="D5" s="49" t="inlineStr"/>

</xml_diff>

<commit_message>
Add VBA integration for PowerPoint presentation management
- Introduced a new Python script `elsagda.py` to handle VBA code generation for PowerPoint presentations.
- Implemented functions to manage slide transitions and custom shows based on section IDs.
- Added error handling for slide navigation and hyperlink actions within the slideshow.
- Integrated Excel data retrieval for dynamic slide content based on seasonal and bishop-specific requirements.
- Enhanced the presentation flow by allowing for guest bishop scenarios with conditional slide management.
- Included binary changes for Excel and PowerPoint files to support the new functionality.
</commit_message>
<xml_diff>
--- a/Tables.xlsx
+++ b/Tables.xlsx
@@ -2677,19 +2677,19 @@
         <v>182</v>
       </c>
       <c r="D10" s="47" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E10" s="47" t="n">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F10" s="47" t="n">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="G10" s="47" t="n">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="H10" s="47" t="n">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="I10" s="43" t="n"/>
     </row>
@@ -2701,22 +2701,22 @@
         <v>8</v>
       </c>
       <c r="C11" s="47" t="n">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D11" s="47" t="n">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="E11" s="47" t="n">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="F11" s="47" t="n">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="G11" s="47" t="n">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="H11" s="47" t="n">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="I11" s="43" t="n"/>
     </row>
@@ -2728,22 +2728,22 @@
         <v>8</v>
       </c>
       <c r="C12" s="47" t="n">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D12" s="47" t="n">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="E12" s="47" t="n">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="F12" s="47" t="n">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="G12" s="47" t="n">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="H12" s="47" t="n">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="I12" s="43" t="n"/>
     </row>
@@ -2755,22 +2755,22 @@
         <v>8</v>
       </c>
       <c r="C13" s="47" t="n">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D13" s="47" t="n">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E13" s="47" t="n">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="F13" s="47" t="n">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="G13" s="47" t="n">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="H13" s="47" t="n">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="I13" s="43" t="n"/>
     </row>
@@ -2782,22 +2782,22 @@
         <v>8</v>
       </c>
       <c r="C14" s="47" t="n">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="D14" s="47" t="n">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E14" s="47" t="n">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="F14" s="47" t="n">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="G14" s="47" t="n">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="H14" s="47" t="n">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="I14" s="43" t="n"/>
     </row>
@@ -2809,22 +2809,22 @@
         <v>8</v>
       </c>
       <c r="C15" s="47" t="n">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="D15" s="47" t="n">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="E15" s="47" t="n">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="F15" s="47" t="n">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="G15" s="47" t="n">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H15" s="47" t="n">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I15" s="43" t="n"/>
     </row>
@@ -2836,22 +2836,22 @@
         <v>8</v>
       </c>
       <c r="C16" s="47" t="n">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="D16" s="47" t="n">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="E16" s="47" t="n">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="F16" s="47" t="n">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="G16" s="47" t="n">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="H16" s="47" t="n">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="I16" s="43" t="n"/>
     </row>
@@ -2863,22 +2863,22 @@
         <v>8</v>
       </c>
       <c r="C17" s="47" t="n">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="D17" s="47" t="n">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="E17" s="47" t="n">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="F17" s="47" t="n">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="G17" s="47" t="n">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="H17" s="47" t="n">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="I17" s="43" t="n"/>
     </row>
@@ -2890,22 +2890,22 @@
         <v>8</v>
       </c>
       <c r="C18" s="47" t="n">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="D18" s="47" t="n">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="E18" s="47" t="n">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="F18" s="47" t="n">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="G18" s="47" t="n">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="H18" s="47" t="n">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="I18" s="43" t="n"/>
     </row>
@@ -2917,22 +2917,22 @@
         <v>8</v>
       </c>
       <c r="C19" s="47" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="D19" s="47" t="n">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="E19" s="47" t="n">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="F19" s="47" t="n">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="G19" s="47" t="n">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="H19" s="47" t="n">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="I19" s="43" t="n"/>
     </row>
@@ -2944,22 +2944,22 @@
         <v>8</v>
       </c>
       <c r="C20" s="47" t="n">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="D20" s="47" t="n">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="E20" s="47" t="n">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="F20" s="47" t="n">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="G20" s="47" t="n">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="H20" s="47" t="n">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="I20" s="43" t="n"/>
     </row>
@@ -2971,22 +2971,22 @@
         <v>8</v>
       </c>
       <c r="C21" s="47" t="n">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="D21" s="47" t="n">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="E21" s="47" t="n">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="F21" s="47" t="n">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G21" s="47" t="n">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="H21" s="47" t="n">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="I21" s="43" t="n"/>
     </row>
@@ -2998,22 +2998,22 @@
         <v>8</v>
       </c>
       <c r="C22" s="47" t="n">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="D22" s="47" t="n">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E22" s="47" t="n">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="F22" s="47" t="n">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="G22" s="47" t="n">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="H22" s="47" t="n">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="I22" s="43" t="n"/>
     </row>
@@ -3025,22 +3025,22 @@
         <v>8</v>
       </c>
       <c r="C23" s="47" t="n">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="D23" s="47" t="n">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="E23" s="47" t="n">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="F23" s="47" t="n">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="G23" s="47" t="n">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="H23" s="47" t="n">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="I23" s="43" t="n"/>
     </row>
@@ -3052,22 +3052,22 @@
         <v>8</v>
       </c>
       <c r="C24" s="47" t="n">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="D24" s="47" t="n">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="E24" s="47" t="n">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="F24" s="47" t="n">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="G24" s="47" t="n">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="H24" s="47" t="n">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="I24" s="43" t="n"/>
     </row>
@@ -3079,22 +3079,22 @@
         <v>8</v>
       </c>
       <c r="C25" s="47" t="n">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="D25" s="47" t="n">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="E25" s="47" t="n">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="F25" s="47" t="n">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="G25" s="47" t="n">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="H25" s="47" t="n">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="I25" s="43" t="n"/>
     </row>
@@ -3106,22 +3106,22 @@
         <v>8</v>
       </c>
       <c r="C26" s="47" t="n">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="D26" s="47" t="n">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="E26" s="47" t="n">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="F26" s="47" t="n">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="G26" s="47" t="n">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="H26" s="47" t="n">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="I26" s="43" t="n"/>
     </row>
@@ -3133,22 +3133,22 @@
         <v>8</v>
       </c>
       <c r="C27" s="47" t="n">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="D27" s="47" t="n">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="E27" s="47" t="n">
-        <v>402</v>
+        <v>407</v>
       </c>
       <c r="F27" s="47" t="n">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="G27" s="47" t="n">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="H27" s="47" t="n">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="I27" s="43" t="n"/>
     </row>
@@ -3160,22 +3160,22 @@
         <v>8</v>
       </c>
       <c r="C28" s="47" t="n">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="D28" s="47" t="n">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="E28" s="47" t="n">
-        <v>414</v>
+        <v>419</v>
       </c>
       <c r="F28" s="47" t="n">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="G28" s="47" t="n">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="H28" s="47" t="n">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="I28" s="43" t="n"/>
     </row>
@@ -3187,22 +3187,22 @@
         <v>9</v>
       </c>
       <c r="C29" s="47" t="n">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="D29" s="47" t="n">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="E29" s="47" t="n">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="F29" s="47" t="n">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="G29" s="47" t="n">
-        <v>434</v>
+        <v>439</v>
       </c>
       <c r="H29" s="47" t="n">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="I29" s="43" t="n"/>
     </row>
@@ -3214,22 +3214,22 @@
         <v>9</v>
       </c>
       <c r="C30" s="47" t="n">
-        <v>439</v>
+        <v>444</v>
       </c>
       <c r="D30" s="47" t="n">
-        <v>443</v>
+        <v>448</v>
       </c>
       <c r="E30" s="47" t="n">
-        <v>446</v>
+        <v>451</v>
       </c>
       <c r="F30" s="47" t="n">
-        <v>453</v>
+        <v>458</v>
       </c>
       <c r="G30" s="47" t="n">
-        <v>454</v>
+        <v>459</v>
       </c>
       <c r="H30" s="47" t="n">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I30" s="43" t="n"/>
     </row>
@@ -3241,22 +3241,22 @@
         <v>9</v>
       </c>
       <c r="C31" s="47" t="n">
-        <v>460</v>
+        <v>465</v>
       </c>
       <c r="D31" s="47" t="n">
-        <v>462</v>
+        <v>467</v>
       </c>
       <c r="E31" s="47" t="n">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="F31" s="47" t="n">
-        <v>467</v>
+        <v>472</v>
       </c>
       <c r="G31" s="47" t="n">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="H31" s="47" t="n">
-        <v>470</v>
+        <v>475</v>
       </c>
       <c r="I31" s="43" t="n"/>
     </row>
@@ -3268,22 +3268,22 @@
         <v>9</v>
       </c>
       <c r="C32" s="47" t="n">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="D32" s="47" t="n">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="E32" s="47" t="n">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="F32" s="47" t="n">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="G32" s="47" t="n">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="H32" s="47" t="n">
-        <v>481</v>
+        <v>486</v>
       </c>
       <c r="I32" s="43" t="n"/>
     </row>
@@ -3295,22 +3295,22 @@
         <v>9</v>
       </c>
       <c r="C33" s="47" t="n">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="D33" s="47" t="n">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="E33" s="47" t="n">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="F33" s="47" t="n">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="G33" s="47" t="n">
-        <v>492</v>
+        <v>497</v>
       </c>
       <c r="H33" s="47" t="n">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="I33" s="43" t="n"/>
     </row>
@@ -3322,22 +3322,22 @@
         <v>9</v>
       </c>
       <c r="C34" s="47" t="n">
-        <v>496</v>
+        <v>501</v>
       </c>
       <c r="D34" s="47" t="n">
-        <v>499</v>
+        <v>504</v>
       </c>
       <c r="E34" s="47" t="n">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="F34" s="47" t="n">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="G34" s="47" t="n">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="H34" s="47" t="n">
-        <v>506</v>
+        <v>511</v>
       </c>
       <c r="I34" s="43" t="n"/>
     </row>
@@ -3349,22 +3349,22 @@
         <v>9</v>
       </c>
       <c r="C35" s="47" t="n">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="D35" s="47" t="n">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="E35" s="47" t="n">
-        <v>512</v>
+        <v>519</v>
       </c>
       <c r="F35" s="47" t="n">
-        <v>513</v>
+        <v>521</v>
       </c>
       <c r="G35" s="47" t="n">
-        <v>514</v>
+        <v>522</v>
       </c>
       <c r="H35" s="47" t="n">
-        <v>515</v>
+        <v>524</v>
       </c>
       <c r="I35" s="43" t="n"/>
     </row>
@@ -3376,22 +3376,22 @@
         <v>9</v>
       </c>
       <c r="C36" s="47" t="n">
-        <v>517</v>
+        <v>526</v>
       </c>
       <c r="D36" s="47" t="n">
-        <v>522</v>
+        <v>532</v>
       </c>
       <c r="E36" s="47" t="n">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="F36" s="47" t="n">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="G36" s="47" t="n">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="H36" s="47" t="n">
-        <v>534</v>
+        <v>546</v>
       </c>
       <c r="I36" s="43" t="n"/>
     </row>
@@ -3403,22 +3403,22 @@
         <v>9</v>
       </c>
       <c r="C37" s="47" t="n">
-        <v>536</v>
+        <v>548</v>
       </c>
       <c r="D37" s="47" t="n">
-        <v>543</v>
+        <v>555</v>
       </c>
       <c r="E37" s="47" t="n">
-        <v>547</v>
+        <v>559</v>
       </c>
       <c r="F37" s="47" t="n">
-        <v>556</v>
+        <v>568</v>
       </c>
       <c r="G37" s="47" t="n">
-        <v>557</v>
+        <v>569</v>
       </c>
       <c r="H37" s="47" t="n">
-        <v>559</v>
+        <v>571</v>
       </c>
       <c r="I37" s="43" t="n"/>
     </row>
@@ -3430,22 +3430,22 @@
         <v>9</v>
       </c>
       <c r="C38" s="47" t="n">
-        <v>561</v>
+        <v>573</v>
       </c>
       <c r="D38" s="47" t="n">
-        <v>563</v>
+        <v>575</v>
       </c>
       <c r="E38" s="47" t="n">
-        <v>566</v>
+        <v>578</v>
       </c>
       <c r="F38" s="47" t="n">
-        <v>569</v>
+        <v>581</v>
       </c>
       <c r="G38" s="47" t="n">
-        <v>570</v>
+        <v>582</v>
       </c>
       <c r="H38" s="47" t="n">
-        <v>574</v>
+        <v>586</v>
       </c>
       <c r="I38" s="43" t="n"/>
     </row>
@@ -3457,22 +3457,22 @@
         <v>9</v>
       </c>
       <c r="C39" s="47" t="n">
-        <v>576</v>
+        <v>588</v>
       </c>
       <c r="D39" s="47" t="n">
-        <v>578</v>
+        <v>590</v>
       </c>
       <c r="E39" s="47" t="n">
-        <v>580</v>
+        <v>592</v>
       </c>
       <c r="F39" s="47" t="n">
-        <v>582</v>
+        <v>594</v>
       </c>
       <c r="G39" s="47" t="n">
-        <v>583</v>
+        <v>595</v>
       </c>
       <c r="H39" s="47" t="n">
-        <v>587</v>
+        <v>599</v>
       </c>
       <c r="I39" s="43" t="n"/>
     </row>
@@ -3484,22 +3484,22 @@
         <v>9</v>
       </c>
       <c r="C40" s="47" t="n">
-        <v>589</v>
+        <v>601</v>
       </c>
       <c r="D40" s="47" t="n">
-        <v>593</v>
+        <v>605</v>
       </c>
       <c r="E40" s="47" t="n">
-        <v>596</v>
+        <v>608</v>
       </c>
       <c r="F40" s="47" t="n">
-        <v>598</v>
+        <v>610</v>
       </c>
       <c r="G40" s="47" t="n">
-        <v>599</v>
+        <v>611</v>
       </c>
       <c r="H40" s="47" t="n">
-        <v>602</v>
+        <v>614</v>
       </c>
       <c r="I40" s="43" t="n"/>
     </row>
@@ -3511,22 +3511,22 @@
         <v>9</v>
       </c>
       <c r="C41" s="8" t="n">
-        <v>604</v>
+        <v>616</v>
       </c>
       <c r="D41" s="8" t="n">
-        <v>606</v>
+        <v>618</v>
       </c>
       <c r="E41" s="8" t="n">
-        <v>611</v>
+        <v>623</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>619</v>
+        <v>631</v>
       </c>
       <c r="G41" s="8" t="n">
-        <v>620</v>
+        <v>632</v>
       </c>
       <c r="H41" s="8" t="n">
-        <v>625</v>
+        <v>637</v>
       </c>
       <c r="I41" s="77" t="inlineStr">
         <is>
@@ -3542,22 +3542,22 @@
         <v>9</v>
       </c>
       <c r="C42" s="47" t="n">
-        <v>627</v>
+        <v>639</v>
       </c>
       <c r="D42" s="47" t="n">
-        <v>634</v>
+        <v>646</v>
       </c>
       <c r="E42" s="47" t="n">
-        <v>638</v>
+        <v>650</v>
       </c>
       <c r="F42" s="47" t="n">
-        <v>640</v>
+        <v>652</v>
       </c>
       <c r="G42" s="47" t="n">
-        <v>641</v>
+        <v>653</v>
       </c>
       <c r="H42" s="47" t="n">
-        <v>643</v>
+        <v>655</v>
       </c>
       <c r="I42" s="77" t="n"/>
     </row>
@@ -3569,22 +3569,22 @@
         <v>9</v>
       </c>
       <c r="C43" s="47" t="n">
-        <v>645</v>
+        <v>657</v>
       </c>
       <c r="D43" s="47" t="n">
-        <v>648</v>
+        <v>660</v>
       </c>
       <c r="E43" s="47" t="n">
-        <v>651</v>
+        <v>663</v>
       </c>
       <c r="F43" s="47" t="n">
-        <v>655</v>
+        <v>667</v>
       </c>
       <c r="G43" s="47" t="n">
-        <v>656</v>
+        <v>668</v>
       </c>
       <c r="H43" s="47" t="n">
-        <v>658</v>
+        <v>670</v>
       </c>
       <c r="I43" s="77" t="n"/>
     </row>
@@ -3596,22 +3596,22 @@
         <v>9</v>
       </c>
       <c r="C44" s="47" t="n">
-        <v>660</v>
+        <v>672</v>
       </c>
       <c r="D44" s="47" t="n">
-        <v>664</v>
+        <v>676</v>
       </c>
       <c r="E44" s="47" t="n">
-        <v>668</v>
+        <v>680</v>
       </c>
       <c r="F44" s="47" t="n">
-        <v>674</v>
+        <v>686</v>
       </c>
       <c r="G44" s="47" t="n">
-        <v>675</v>
+        <v>687</v>
       </c>
       <c r="H44" s="47" t="n">
-        <v>678</v>
+        <v>690</v>
       </c>
       <c r="I44" s="77" t="n"/>
     </row>
@@ -3623,22 +3623,22 @@
         <v>9</v>
       </c>
       <c r="C45" s="47" t="n">
-        <v>680</v>
+        <v>692</v>
       </c>
       <c r="D45" s="47" t="n">
-        <v>683</v>
+        <v>695</v>
       </c>
       <c r="E45" s="47" t="n">
-        <v>688</v>
+        <v>700</v>
       </c>
       <c r="F45" s="47" t="n">
-        <v>691</v>
+        <v>703</v>
       </c>
       <c r="G45" s="47" t="n">
-        <v>692</v>
+        <v>704</v>
       </c>
       <c r="H45" s="47" t="n">
-        <v>694</v>
+        <v>706</v>
       </c>
       <c r="I45" s="77" t="n"/>
     </row>
@@ -3650,22 +3650,22 @@
         <v>9</v>
       </c>
       <c r="C46" s="47" t="n">
-        <v>696</v>
+        <v>708</v>
       </c>
       <c r="D46" s="47" t="n">
-        <v>699</v>
+        <v>711</v>
       </c>
       <c r="E46" s="47" t="n">
-        <v>703</v>
+        <v>715</v>
       </c>
       <c r="F46" s="47" t="n">
-        <v>705</v>
+        <v>717</v>
       </c>
       <c r="G46" s="47" t="n">
-        <v>706</v>
+        <v>718</v>
       </c>
       <c r="H46" s="47" t="n">
-        <v>707</v>
+        <v>719</v>
       </c>
       <c r="I46" s="77" t="n"/>
     </row>
@@ -3677,22 +3677,22 @@
         <v>9</v>
       </c>
       <c r="C47" s="47" t="n">
-        <v>709</v>
+        <v>721</v>
       </c>
       <c r="D47" s="47" t="n">
-        <v>715</v>
+        <v>727</v>
       </c>
       <c r="E47" s="47" t="n">
-        <v>719</v>
+        <v>731</v>
       </c>
       <c r="F47" s="47" t="n">
-        <v>722</v>
+        <v>734</v>
       </c>
       <c r="G47" s="47" t="n">
-        <v>723</v>
+        <v>735</v>
       </c>
       <c r="H47" s="47" t="n">
-        <v>724</v>
+        <v>736</v>
       </c>
       <c r="I47" s="77" t="n"/>
     </row>
@@ -3704,22 +3704,22 @@
         <v>9</v>
       </c>
       <c r="C48" s="47" t="n">
-        <v>726</v>
+        <v>738</v>
       </c>
       <c r="D48" s="47" t="n">
-        <v>731</v>
+        <v>743</v>
       </c>
       <c r="E48" s="47" t="n">
-        <v>734</v>
+        <v>746</v>
       </c>
       <c r="F48" s="47" t="n">
-        <v>737</v>
+        <v>749</v>
       </c>
       <c r="G48" s="47" t="n">
-        <v>738</v>
+        <v>750</v>
       </c>
       <c r="H48" s="47" t="n">
-        <v>740</v>
+        <v>752</v>
       </c>
       <c r="I48" s="77" t="n"/>
     </row>
@@ -3731,22 +3731,22 @@
         <v>9</v>
       </c>
       <c r="C49" s="47" t="n">
-        <v>742</v>
+        <v>754</v>
       </c>
       <c r="D49" s="47" t="n">
-        <v>745</v>
+        <v>757</v>
       </c>
       <c r="E49" s="47" t="n">
-        <v>747</v>
+        <v>759</v>
       </c>
       <c r="F49" s="47" t="n">
-        <v>749</v>
+        <v>761</v>
       </c>
       <c r="G49" s="47" t="n">
-        <v>750</v>
+        <v>762</v>
       </c>
       <c r="H49" s="47" t="n">
-        <v>751</v>
+        <v>763</v>
       </c>
       <c r="I49" s="77" t="n"/>
     </row>
@@ -3758,22 +3758,22 @@
         <v>9</v>
       </c>
       <c r="C50" s="47" t="n">
-        <v>753</v>
+        <v>765</v>
       </c>
       <c r="D50" s="47" t="n">
-        <v>761</v>
+        <v>773</v>
       </c>
       <c r="E50" s="47" t="n">
-        <v>765</v>
+        <v>777</v>
       </c>
       <c r="F50" s="47" t="n">
-        <v>772</v>
+        <v>784</v>
       </c>
       <c r="G50" s="47" t="n">
-        <v>773</v>
+        <v>785</v>
       </c>
       <c r="H50" s="47" t="n">
-        <v>777</v>
+        <v>789</v>
       </c>
       <c r="I50" s="77" t="n"/>
     </row>
@@ -3785,22 +3785,22 @@
         <v>9</v>
       </c>
       <c r="C51" s="8" t="n">
-        <v>779</v>
+        <v>791</v>
       </c>
       <c r="D51" s="8" t="n">
-        <v>792</v>
+        <v>804</v>
       </c>
       <c r="E51" s="8" t="n">
-        <v>797</v>
+        <v>809</v>
       </c>
       <c r="F51" s="8" t="n">
-        <v>806</v>
+        <v>818</v>
       </c>
       <c r="G51" s="8" t="n">
-        <v>807</v>
+        <v>819</v>
       </c>
       <c r="H51" s="8" t="n">
-        <v>813</v>
+        <v>825</v>
       </c>
       <c r="I51" s="77" t="inlineStr">
         <is>
@@ -18283,8 +18283,8 @@
       <c r="B3" s="47" t="n">
         <v>5</v>
       </c>
-      <c r="C3" s="47" t="n"/>
-      <c r="D3" s="47" t="n"/>
+      <c r="C3" s="47" t="inlineStr"/>
+      <c r="D3" s="47" t="inlineStr"/>
       <c r="E3" s="47" t="n"/>
       <c r="F3" s="47" t="n">
         <v>45</v>
@@ -18324,8 +18324,8 @@
       <c r="B4" s="47" t="n">
         <v>5</v>
       </c>
-      <c r="C4" s="47" t="n"/>
-      <c r="D4" s="47" t="n"/>
+      <c r="C4" s="47" t="inlineStr"/>
+      <c r="D4" s="47" t="inlineStr"/>
       <c r="E4" s="47" t="n"/>
       <c r="F4" s="47" t="n">
         <v>71</v>
@@ -18365,10 +18365,10 @@
       <c r="B5" s="47" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="47" t="n"/>
-      <c r="D5" s="47" t="n"/>
+      <c r="C5" s="47" t="inlineStr"/>
+      <c r="D5" s="47" t="inlineStr"/>
       <c r="E5" s="47" t="n"/>
-      <c r="F5" s="47" t="n"/>
+      <c r="F5" s="47" t="inlineStr"/>
       <c r="G5" s="47" t="n">
         <v>107</v>
       </c>

</xml_diff>